<commit_message>
TC_003 Script Updated and Optimized
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BD2F52-22CB-4346-B8C9-2B3FDCBDD5E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5B6448-B315-46DE-B516-E51F6474F972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="3" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="68">
   <si>
     <t>Username</t>
   </si>
@@ -215,6 +215,24 @@
   </si>
   <si>
     <t>Kochukhet, Kafrul, Dhaka, Dhaka Metropolitan, Dhaka District, Dhaka Division, 1103, Bangladesh</t>
+  </si>
+  <si>
+    <t>1-2</t>
+  </si>
+  <si>
+    <t>rokybul.imrose@savethechildren.org</t>
+  </si>
+  <si>
+    <t>Mohakhali, Bir Uttam A. K. Khandakar Road, Gulshan 1, Mohakhali, Dhaka, Dhaka Metropolitan, Dhaka District, Dhaka Division, 1213, Bangladesh</t>
+  </si>
+  <si>
+    <t>Rajshahi</t>
+  </si>
+  <si>
+    <t>Rongpur</t>
+  </si>
+  <si>
+    <t>1-4</t>
   </si>
 </sst>
 </file>
@@ -244,7 +262,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -272,6 +290,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -328,11 +352,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -360,14 +381,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -392,7 +409,20 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -733,92 +763,92 @@
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.6328125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="7.54296875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="15.26953125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="57.26953125" style="17" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="17"/>
+    <col min="1" max="1" width="11.6328125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="7.54296875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="15.26953125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="57.26953125" style="14" customWidth="1"/>
+    <col min="5" max="16384" width="8.7265625" style="14"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="3">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="15" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="15" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="15" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3">
         <v>4</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="15" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3">
         <v>5</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="18"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="15"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3">
         <v>6</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="18"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="15"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -836,74 +866,74 @@
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.08984375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="8.54296875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="11.08984375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="10.6328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.90625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.7265625" style="3"/>
+    <col min="1" max="1" width="11.08984375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="8.54296875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="11.08984375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.6328125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.90625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="13" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="3">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>12345</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F2" s="16" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3">
         <v>2</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="17"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3">
         <v>3</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="20"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="17"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -916,64 +946,64 @@
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.08984375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="7.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="11.08984375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="10.6328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="3"/>
+    <col min="1" max="1" width="11.08984375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="7.6328125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="11.08984375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.6328125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="D1" s="19" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="3">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>12345</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3">
         <v>2</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3">
         <v>3</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3">
         <v>4</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -982,263 +1012,295 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC28C683-2DE1-4543-8063-C85149D9A2B2}">
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.81640625" style="9" customWidth="1"/>
-    <col min="2" max="2" width="5.6328125" style="9" customWidth="1"/>
-    <col min="3" max="4" width="8.7265625" style="9"/>
-    <col min="5" max="5" width="13.36328125" style="9" customWidth="1"/>
-    <col min="6" max="7" width="15.36328125" style="9" customWidth="1"/>
-    <col min="8" max="9" width="8.7265625" style="9"/>
-    <col min="10" max="10" width="15.08984375" style="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.08984375" style="12" customWidth="1"/>
-    <col min="12" max="12" width="8.7265625" style="9"/>
-    <col min="13" max="13" width="10.81640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="14" max="16" width="8.7265625" style="9"/>
-    <col min="17" max="17" width="10.81640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="8.7265625" style="9"/>
+    <col min="1" max="1" width="11.81640625" style="10" customWidth="1"/>
+    <col min="2" max="2" width="5.6328125" style="10" customWidth="1"/>
+    <col min="3" max="4" width="8.7265625" style="10"/>
+    <col min="5" max="5" width="13.36328125" style="10" customWidth="1"/>
+    <col min="6" max="7" width="15.36328125" style="10" customWidth="1"/>
+    <col min="8" max="9" width="8.7265625" style="10"/>
+    <col min="10" max="10" width="15.08984375" style="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.08984375" style="10" customWidth="1"/>
+    <col min="12" max="12" width="8.7265625" style="10"/>
+    <col min="13" max="13" width="10.81640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="8.7265625" style="10"/>
+    <col min="17" max="17" width="10.81640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="8.7265625" style="10"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="Q1" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="R1" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="S1" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="T1" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="U1" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="V1" s="6" t="s">
+      <c r="V1" s="7" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="116" x14ac:dyDescent="0.35">
-      <c r="A2" s="2">
+      <c r="A2" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="9">
         <v>1</v>
       </c>
-      <c r="B2" s="2">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="9">
         <v>12345</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="J2" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="K2" s="10" t="s">
+      <c r="K2" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M2" s="11" t="s">
+      <c r="M2" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="O2" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="P2" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="Q2" s="11" t="s">
+      <c r="Q2" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="R2" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="S2" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="T2" s="2">
+      <c r="T2" s="9">
         <v>50</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="U2" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="V2" s="2" t="s">
+      <c r="V2" s="9" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2">
+    <row r="3" spans="1:22" ht="145" x14ac:dyDescent="0.35">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9">
         <v>2</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="9"/>
+      <c r="T3" s="9"/>
+      <c r="U3" s="9"/>
+      <c r="V3" s="9"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9">
         <v>3</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
-      <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
+      <c r="P4" s="9"/>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9"/>
+      <c r="S4" s="9"/>
+      <c r="T4" s="9"/>
+      <c r="U4" s="9"/>
+      <c r="V4" s="9"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2">
+      <c r="A5" s="9"/>
+      <c r="B5" s="9">
         <v>4</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="10"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
-      <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="9"/>
+      <c r="P5" s="9"/>
+      <c r="Q5" s="9"/>
+      <c r="R5" s="9"/>
+      <c r="S5" s="9"/>
+      <c r="T5" s="9"/>
+      <c r="U5" s="9"/>
+      <c r="V5" s="9"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9">
         <v>5</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="2"/>
-      <c r="T6" s="2"/>
-      <c r="U6" s="2"/>
-      <c r="V6" s="2"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
+      <c r="P6" s="9"/>
+      <c r="Q6" s="9"/>
+      <c r="R6" s="9"/>
+      <c r="S6" s="9"/>
+      <c r="T6" s="9"/>
+      <c r="U6" s="9"/>
+      <c r="V6" s="9"/>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A7" s="9"/>
+      <c r="B7" s="9">
+        <v>6</v>
+      </c>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="9"/>
+      <c r="P7" s="9"/>
+      <c r="Q7" s="9"/>
+      <c r="R7" s="9"/>
+      <c r="S7" s="9"/>
+      <c r="T7" s="9"/>
+      <c r="U7" s="9"/>
+      <c r="V7" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1247,151 +1309,197 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B1CFC64-F19E-4BC4-A1E5-2FDFF8A8F1BB}">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.7265625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="10.90625" style="3" customWidth="1"/>
-    <col min="3" max="4" width="13.26953125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="30.6328125" style="3" customWidth="1"/>
-    <col min="6" max="7" width="19.54296875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="35" style="3" customWidth="1"/>
-    <col min="9" max="9" width="17.26953125" style="3" customWidth="1"/>
-    <col min="10" max="10" width="17.90625" style="3" customWidth="1"/>
-    <col min="11" max="16384" width="8.7265625" style="3"/>
+    <col min="1" max="1" width="10.7265625" style="10" customWidth="1"/>
+    <col min="2" max="2" width="10.7265625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="10.90625" style="8" customWidth="1"/>
+    <col min="4" max="5" width="13.26953125" style="8" customWidth="1"/>
+    <col min="6" max="6" width="30.6328125" style="8" customWidth="1"/>
+    <col min="7" max="8" width="19.54296875" style="8" customWidth="1"/>
+    <col min="9" max="9" width="35" style="8" customWidth="1"/>
+    <col min="10" max="10" width="17.26953125" style="8" customWidth="1"/>
+    <col min="11" max="11" width="17.90625" style="8" customWidth="1"/>
+    <col min="12" max="16384" width="8.7265625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1">
+        <v>12345</v>
+      </c>
+      <c r="E2" s="1">
+        <v>830</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="1">
+        <v>12345</v>
+      </c>
+      <c r="H2" s="1">
+        <v>872</v>
+      </c>
+      <c r="I2" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="J2" s="1">
+        <v>12345</v>
+      </c>
+      <c r="K2" s="1">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" s="9"/>
+      <c r="B3" s="1">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1">
+        <v>12345</v>
+      </c>
+      <c r="E3" s="1">
+        <v>830</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G3" s="1">
+        <v>12345</v>
+      </c>
+      <c r="H3" s="1">
+        <v>872</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="J3" s="1">
+        <v>12345</v>
+      </c>
+      <c r="K3" s="1">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" s="9"/>
+      <c r="B4" s="1">
         <v>3</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4">
+      <c r="D4" s="1">
         <v>12345</v>
       </c>
-      <c r="D2" s="4">
-        <v>830</v>
-      </c>
-      <c r="E2" s="14" t="s">
+      <c r="E4" s="1">
+        <v>831</v>
+      </c>
+      <c r="F4" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="2">
+      <c r="G4" s="1">
         <v>12345</v>
       </c>
-      <c r="G2" s="4">
-        <v>872</v>
-      </c>
-      <c r="H2" s="14" t="s">
+      <c r="H4" s="1">
+        <v>873</v>
+      </c>
+      <c r="I4" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="I2" s="2">
+      <c r="J4" s="1">
         <v>12345</v>
       </c>
-      <c r="J2" s="4">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4" t="s">
+      <c r="K4" s="1">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="9"/>
+      <c r="B5" s="1">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="4">
+      <c r="D5" s="1">
         <v>12345</v>
       </c>
-      <c r="D3" s="4">
-        <v>831</v>
-      </c>
-      <c r="E3" s="13" t="s">
+      <c r="E5" s="1">
+        <v>832</v>
+      </c>
+      <c r="F5" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="F3" s="2">
+      <c r="G5" s="1">
         <v>12345</v>
       </c>
-      <c r="G3" s="4">
-        <v>873</v>
-      </c>
-      <c r="H3" s="13" t="s">
+      <c r="H5" s="1">
+        <v>874</v>
+      </c>
+      <c r="I5" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="I3" s="2">
+      <c r="J5" s="1">
         <v>12345</v>
       </c>
-      <c r="J3" s="4">
-        <v>873</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="4">
-        <v>12345</v>
-      </c>
-      <c r="D4" s="4">
-        <v>832</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="F4" s="2">
-        <v>12345</v>
-      </c>
-      <c r="G4" s="4">
+      <c r="K5" s="1">
         <v>874</v>
       </c>
-      <c r="H4" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="I4" s="2">
-        <v>12345</v>
-      </c>
-      <c r="J4" s="4">
-        <v>874</v>
-      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="E3:E4" r:id="rId1" display="mohi.uddin@savethechildren.org" xr:uid="{B86BD464-751E-49E0-A260-F8A19C0DE86F}"/>
-    <hyperlink ref="H3:H4" r:id="rId2" display="shyamal.mondal@savethechildren.org" xr:uid="{48C7FCC0-A8F3-43C1-99E4-D4F4592D9DBE}"/>
-    <hyperlink ref="E2" r:id="rId3" xr:uid="{2FA4BAB4-A9A9-4756-89D1-21AD392C38D1}"/>
-    <hyperlink ref="H2" r:id="rId4" xr:uid="{27B85803-F778-4639-AB02-9C77547AFEBB}"/>
+    <hyperlink ref="F3" r:id="rId1" xr:uid="{D6323319-3F75-49A5-9F15-EF38138D42B0}"/>
+    <hyperlink ref="I3" r:id="rId2" xr:uid="{FCD8BB58-86CE-41E3-97AC-B55E5F8271F4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
TC_004 is in progress
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BD2F52-22CB-4346-B8C9-2B3FDCBDD5E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5B6448-B315-46DE-B516-E51F6474F972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="3" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="68">
   <si>
     <t>Username</t>
   </si>
@@ -215,6 +215,24 @@
   </si>
   <si>
     <t>Kochukhet, Kafrul, Dhaka, Dhaka Metropolitan, Dhaka District, Dhaka Division, 1103, Bangladesh</t>
+  </si>
+  <si>
+    <t>1-2</t>
+  </si>
+  <si>
+    <t>rokybul.imrose@savethechildren.org</t>
+  </si>
+  <si>
+    <t>Mohakhali, Bir Uttam A. K. Khandakar Road, Gulshan 1, Mohakhali, Dhaka, Dhaka Metropolitan, Dhaka District, Dhaka Division, 1213, Bangladesh</t>
+  </si>
+  <si>
+    <t>Rajshahi</t>
+  </si>
+  <si>
+    <t>Rongpur</t>
+  </si>
+  <si>
+    <t>1-4</t>
   </si>
 </sst>
 </file>
@@ -244,7 +262,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -272,6 +290,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -328,11 +352,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -360,14 +381,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -392,7 +409,20 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -733,92 +763,92 @@
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.6328125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="7.54296875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="15.26953125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="57.26953125" style="17" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="17"/>
+    <col min="1" max="1" width="11.6328125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="7.54296875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="15.26953125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="57.26953125" style="14" customWidth="1"/>
+    <col min="5" max="16384" width="8.7265625" style="14"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="3">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="15" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="15" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="15" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3">
         <v>4</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="15" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3">
         <v>5</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="18"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="15"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3">
         <v>6</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="18"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="15"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -836,74 +866,74 @@
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.08984375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="8.54296875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="11.08984375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="10.6328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.90625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.7265625" style="3"/>
+    <col min="1" max="1" width="11.08984375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="8.54296875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="11.08984375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.6328125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.90625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="13" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="3">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>12345</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F2" s="16" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3">
         <v>2</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="17"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3">
         <v>3</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="20"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="17"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -916,64 +946,64 @@
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.08984375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="7.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="11.08984375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="10.6328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="3"/>
+    <col min="1" max="1" width="11.08984375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="7.6328125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="11.08984375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.6328125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="D1" s="19" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="3">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>12345</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3">
         <v>2</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3">
         <v>3</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3">
         <v>4</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -982,263 +1012,295 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC28C683-2DE1-4543-8063-C85149D9A2B2}">
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.81640625" style="9" customWidth="1"/>
-    <col min="2" max="2" width="5.6328125" style="9" customWidth="1"/>
-    <col min="3" max="4" width="8.7265625" style="9"/>
-    <col min="5" max="5" width="13.36328125" style="9" customWidth="1"/>
-    <col min="6" max="7" width="15.36328125" style="9" customWidth="1"/>
-    <col min="8" max="9" width="8.7265625" style="9"/>
-    <col min="10" max="10" width="15.08984375" style="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.08984375" style="12" customWidth="1"/>
-    <col min="12" max="12" width="8.7265625" style="9"/>
-    <col min="13" max="13" width="10.81640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="14" max="16" width="8.7265625" style="9"/>
-    <col min="17" max="17" width="10.81640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="8.7265625" style="9"/>
+    <col min="1" max="1" width="11.81640625" style="10" customWidth="1"/>
+    <col min="2" max="2" width="5.6328125" style="10" customWidth="1"/>
+    <col min="3" max="4" width="8.7265625" style="10"/>
+    <col min="5" max="5" width="13.36328125" style="10" customWidth="1"/>
+    <col min="6" max="7" width="15.36328125" style="10" customWidth="1"/>
+    <col min="8" max="9" width="8.7265625" style="10"/>
+    <col min="10" max="10" width="15.08984375" style="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.08984375" style="10" customWidth="1"/>
+    <col min="12" max="12" width="8.7265625" style="10"/>
+    <col min="13" max="13" width="10.81640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="8.7265625" style="10"/>
+    <col min="17" max="17" width="10.81640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="8.7265625" style="10"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="Q1" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="R1" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="S1" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="T1" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="U1" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="V1" s="6" t="s">
+      <c r="V1" s="7" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="116" x14ac:dyDescent="0.35">
-      <c r="A2" s="2">
+      <c r="A2" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="9">
         <v>1</v>
       </c>
-      <c r="B2" s="2">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="9">
         <v>12345</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="J2" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="K2" s="10" t="s">
+      <c r="K2" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M2" s="11" t="s">
+      <c r="M2" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="O2" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="P2" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="Q2" s="11" t="s">
+      <c r="Q2" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="R2" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="S2" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="T2" s="2">
+      <c r="T2" s="9">
         <v>50</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="U2" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="V2" s="2" t="s">
+      <c r="V2" s="9" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2">
+    <row r="3" spans="1:22" ht="145" x14ac:dyDescent="0.35">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9">
         <v>2</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="9"/>
+      <c r="T3" s="9"/>
+      <c r="U3" s="9"/>
+      <c r="V3" s="9"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9">
         <v>3</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
-      <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
+      <c r="P4" s="9"/>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9"/>
+      <c r="S4" s="9"/>
+      <c r="T4" s="9"/>
+      <c r="U4" s="9"/>
+      <c r="V4" s="9"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2">
+      <c r="A5" s="9"/>
+      <c r="B5" s="9">
         <v>4</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="10"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
-      <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="9"/>
+      <c r="P5" s="9"/>
+      <c r="Q5" s="9"/>
+      <c r="R5" s="9"/>
+      <c r="S5" s="9"/>
+      <c r="T5" s="9"/>
+      <c r="U5" s="9"/>
+      <c r="V5" s="9"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9">
         <v>5</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="2"/>
-      <c r="T6" s="2"/>
-      <c r="U6" s="2"/>
-      <c r="V6" s="2"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
+      <c r="P6" s="9"/>
+      <c r="Q6" s="9"/>
+      <c r="R6" s="9"/>
+      <c r="S6" s="9"/>
+      <c r="T6" s="9"/>
+      <c r="U6" s="9"/>
+      <c r="V6" s="9"/>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A7" s="9"/>
+      <c r="B7" s="9">
+        <v>6</v>
+      </c>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="9"/>
+      <c r="P7" s="9"/>
+      <c r="Q7" s="9"/>
+      <c r="R7" s="9"/>
+      <c r="S7" s="9"/>
+      <c r="T7" s="9"/>
+      <c r="U7" s="9"/>
+      <c r="V7" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1247,151 +1309,197 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B1CFC64-F19E-4BC4-A1E5-2FDFF8A8F1BB}">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.7265625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="10.90625" style="3" customWidth="1"/>
-    <col min="3" max="4" width="13.26953125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="30.6328125" style="3" customWidth="1"/>
-    <col min="6" max="7" width="19.54296875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="35" style="3" customWidth="1"/>
-    <col min="9" max="9" width="17.26953125" style="3" customWidth="1"/>
-    <col min="10" max="10" width="17.90625" style="3" customWidth="1"/>
-    <col min="11" max="16384" width="8.7265625" style="3"/>
+    <col min="1" max="1" width="10.7265625" style="10" customWidth="1"/>
+    <col min="2" max="2" width="10.7265625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="10.90625" style="8" customWidth="1"/>
+    <col min="4" max="5" width="13.26953125" style="8" customWidth="1"/>
+    <col min="6" max="6" width="30.6328125" style="8" customWidth="1"/>
+    <col min="7" max="8" width="19.54296875" style="8" customWidth="1"/>
+    <col min="9" max="9" width="35" style="8" customWidth="1"/>
+    <col min="10" max="10" width="17.26953125" style="8" customWidth="1"/>
+    <col min="11" max="11" width="17.90625" style="8" customWidth="1"/>
+    <col min="12" max="16384" width="8.7265625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="4">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1">
+        <v>12345</v>
+      </c>
+      <c r="E2" s="1">
+        <v>830</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="1">
+        <v>12345</v>
+      </c>
+      <c r="H2" s="1">
+        <v>872</v>
+      </c>
+      <c r="I2" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="J2" s="1">
+        <v>12345</v>
+      </c>
+      <c r="K2" s="1">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" s="9"/>
+      <c r="B3" s="1">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1">
+        <v>12345</v>
+      </c>
+      <c r="E3" s="1">
+        <v>830</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G3" s="1">
+        <v>12345</v>
+      </c>
+      <c r="H3" s="1">
+        <v>872</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="J3" s="1">
+        <v>12345</v>
+      </c>
+      <c r="K3" s="1">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" s="9"/>
+      <c r="B4" s="1">
         <v>3</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4">
+      <c r="D4" s="1">
         <v>12345</v>
       </c>
-      <c r="D2" s="4">
-        <v>830</v>
-      </c>
-      <c r="E2" s="14" t="s">
+      <c r="E4" s="1">
+        <v>831</v>
+      </c>
+      <c r="F4" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="2">
+      <c r="G4" s="1">
         <v>12345</v>
       </c>
-      <c r="G2" s="4">
-        <v>872</v>
-      </c>
-      <c r="H2" s="14" t="s">
+      <c r="H4" s="1">
+        <v>873</v>
+      </c>
+      <c r="I4" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="I2" s="2">
+      <c r="J4" s="1">
         <v>12345</v>
       </c>
-      <c r="J2" s="4">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4" t="s">
+      <c r="K4" s="1">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="9"/>
+      <c r="B5" s="1">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="4">
+      <c r="D5" s="1">
         <v>12345</v>
       </c>
-      <c r="D3" s="4">
-        <v>831</v>
-      </c>
-      <c r="E3" s="13" t="s">
+      <c r="E5" s="1">
+        <v>832</v>
+      </c>
+      <c r="F5" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="F3" s="2">
+      <c r="G5" s="1">
         <v>12345</v>
       </c>
-      <c r="G3" s="4">
-        <v>873</v>
-      </c>
-      <c r="H3" s="13" t="s">
+      <c r="H5" s="1">
+        <v>874</v>
+      </c>
+      <c r="I5" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="I3" s="2">
+      <c r="J5" s="1">
         <v>12345</v>
       </c>
-      <c r="J3" s="4">
-        <v>873</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="4">
-        <v>12345</v>
-      </c>
-      <c r="D4" s="4">
-        <v>832</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="F4" s="2">
-        <v>12345</v>
-      </c>
-      <c r="G4" s="4">
+      <c r="K5" s="1">
         <v>874</v>
       </c>
-      <c r="H4" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="I4" s="2">
-        <v>12345</v>
-      </c>
-      <c r="J4" s="4">
-        <v>874</v>
-      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="E3:E4" r:id="rId1" display="mohi.uddin@savethechildren.org" xr:uid="{B86BD464-751E-49E0-A260-F8A19C0DE86F}"/>
-    <hyperlink ref="H3:H4" r:id="rId2" display="shyamal.mondal@savethechildren.org" xr:uid="{48C7FCC0-A8F3-43C1-99E4-D4F4592D9DBE}"/>
-    <hyperlink ref="E2" r:id="rId3" xr:uid="{2FA4BAB4-A9A9-4756-89D1-21AD392C38D1}"/>
-    <hyperlink ref="H2" r:id="rId4" xr:uid="{27B85803-F778-4639-AB02-9C77547AFEBB}"/>
+    <hyperlink ref="F3" r:id="rId1" xr:uid="{D6323319-3F75-49A5-9F15-EF38138D42B0}"/>
+    <hyperlink ref="I3" r:id="rId2" xr:uid="{FCD8BB58-86CE-41E3-97AC-B55E5F8271F4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
TC_004 inprogress and script updated
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5B6448-B315-46DE-B516-E51F6474F972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75026ED0-C29D-4B67-8B48-5253F3000EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="3" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="4" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
   <sheets>
     <sheet name="BrowserSetup" sheetId="3" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="68">
   <si>
     <t>Username</t>
   </si>
@@ -1399,15 +1399,9 @@
       <c r="B3" s="1">
         <v>2</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="1">
-        <v>12345</v>
-      </c>
-      <c r="E3" s="1">
-        <v>830</v>
-      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
       <c r="F3" s="11" t="s">
         <v>63</v>
       </c>

</xml_diff>

<commit_message>
TC_004 TS_001 is done
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0421A41E-41D1-4FFF-9B85-BBE23527D94A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6545B097-5AD4-43EC-A7EC-084ED1A1A216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="4" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
+    <workbookView xWindow="720" yWindow="720" windowWidth="17610" windowHeight="8570" tabRatio="902" activeTab="4" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
   <sheets>
     <sheet name="BrowserSetup" sheetId="3" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="64">
   <si>
     <t>Username</t>
   </si>
@@ -88,9 +88,6 @@
     <t>Tania Sharmin</t>
   </si>
   <si>
-    <t>Muhammad Ashik Hassan</t>
-  </si>
-  <si>
     <t>otherSCIPassenger</t>
   </si>
   <si>
@@ -106,9 +103,6 @@
     <t>nonSCIPassengerPhone</t>
   </si>
   <si>
-    <t>Test SOF</t>
-  </si>
-  <si>
     <t>Furniture</t>
   </si>
   <si>
@@ -163,15 +157,6 @@
     <t>InvalidPassword</t>
   </si>
   <si>
-    <t>UserName</t>
-  </si>
-  <si>
-    <t>UserPassword</t>
-  </si>
-  <si>
-    <t>BudgetHolderUserName</t>
-  </si>
-  <si>
     <t>BudgetHolderPassword</t>
   </si>
   <si>
@@ -181,15 +166,6 @@
     <t>SupervisorPassword</t>
   </si>
   <si>
-    <t>BudgetHolderTripId</t>
-  </si>
-  <si>
-    <t>SupervisorTripId</t>
-  </si>
-  <si>
-    <t>UserTripId</t>
-  </si>
-  <si>
     <t>BrowserName</t>
   </si>
   <si>
@@ -233,6 +209,18 @@
   </si>
   <si>
     <t>1-4</t>
+  </si>
+  <si>
+    <t>Shyamal Kumar Mondal</t>
+  </si>
+  <si>
+    <t>Test Automation SOF</t>
+  </si>
+  <si>
+    <t>TripId</t>
+  </si>
+  <si>
+    <t>BudgetHolderUsername</t>
   </si>
 </sst>
 </file>
@@ -352,7 +340,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -384,7 +372,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -423,6 +410,10 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -766,19 +757,19 @@
     <col min="1" max="1" width="11.6328125" style="2" customWidth="1"/>
     <col min="2" max="2" width="7.54296875" style="2" customWidth="1"/>
     <col min="3" max="3" width="15.26953125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="57.26953125" style="14" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="14"/>
+    <col min="4" max="4" width="57.26953125" style="13" customWidth="1"/>
+    <col min="5" max="16384" width="8.7265625" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="18" t="s">
-        <v>59</v>
+      <c r="B1" s="17" t="s">
+        <v>51</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>2</v>
@@ -792,10 +783,10 @@
         <v>1</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>58</v>
+        <v>48</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -804,9 +795,9 @@
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D3" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>3</v>
       </c>
     </row>
@@ -816,10 +807,10 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>58</v>
+        <v>49</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -828,9 +819,9 @@
         <v>4</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D5" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" s="14" t="s">
         <v>3</v>
       </c>
     </row>
@@ -840,7 +831,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="3"/>
-      <c r="D6" s="15"/>
+      <c r="D6" s="14"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
@@ -848,7 +839,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="15"/>
+      <c r="D7" s="14"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -876,11 +867,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="18" t="s">
-        <v>59</v>
+      <c r="B1" s="17" t="s">
+        <v>51</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>0</v>
@@ -889,10 +880,10 @@
         <v>1</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>43</v>
+        <v>40</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -909,10 +900,10 @@
         <v>12345</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="F2" s="16" t="s">
-        <v>55</v>
+        <v>46</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -923,7 +914,7 @@
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
-      <c r="F3" s="17"/>
+      <c r="F3" s="16"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="3"/>
@@ -933,7 +924,7 @@
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
-      <c r="F4" s="17"/>
+      <c r="F4" s="16"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -954,16 +945,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="C1" s="19" t="s">
+      <c r="B1" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="18" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1031,14 +1022,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="24" t="s">
-        <v>59</v>
+      <c r="B1" s="23" t="s">
+        <v>51</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>6</v>
@@ -1050,13 +1041,13 @@
         <v>8</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J1" s="7" t="s">
         <v>11</v>
@@ -1074,33 +1065,33 @@
         <v>15</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q1" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="R1" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="S1" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="T1" s="7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="U1" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="V1" s="7" t="s">
         <v>28</v>
-      </c>
-      <c r="V1" s="7" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="116" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B2" s="9">
         <v>1</v>
@@ -1118,7 +1109,7 @@
         <v>10</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="H2" s="9" t="s">
         <v>16</v>
@@ -1127,43 +1118,43 @@
         <v>17</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="L2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="M2" s="25" t="s">
-        <v>38</v>
+      <c r="M2" s="24" t="s">
+        <v>36</v>
       </c>
       <c r="N2" s="9" t="s">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="P2" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q2" s="25" t="s">
-        <v>38</v>
+        <v>22</v>
+      </c>
+      <c r="Q2" s="24" t="s">
+        <v>36</v>
       </c>
       <c r="R2" s="9" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="S2" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="T2" s="9">
         <v>50</v>
       </c>
       <c r="U2" s="9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="V2" s="9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:22" ht="145" x14ac:dyDescent="0.35">
@@ -1176,7 +1167,7 @@
       <c r="E3" s="9"/>
       <c r="F3" s="9"/>
       <c r="G3" s="9" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="H3" s="9"/>
       <c r="I3" s="9"/>
@@ -1204,7 +1195,7 @@
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
       <c r="G4" s="9" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
@@ -1232,7 +1223,7 @@
       <c r="E5" s="9"/>
       <c r="F5" s="9"/>
       <c r="G5" s="9" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>
@@ -1309,191 +1300,104 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B1CFC64-F19E-4BC4-A1E5-2FDFF8A8F1BB}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.7265625" style="10" customWidth="1"/>
-    <col min="2" max="2" width="10.7265625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="10.90625" style="8" customWidth="1"/>
-    <col min="4" max="5" width="13.26953125" style="8" customWidth="1"/>
-    <col min="6" max="6" width="30.6328125" style="8" customWidth="1"/>
-    <col min="7" max="8" width="19.54296875" style="8" customWidth="1"/>
-    <col min="9" max="9" width="35" style="8" customWidth="1"/>
-    <col min="10" max="10" width="17.26953125" style="8" customWidth="1"/>
-    <col min="11" max="11" width="17.90625" style="8" customWidth="1"/>
-    <col min="12" max="16384" width="8.7265625" style="8"/>
+    <col min="2" max="3" width="10.7265625" style="8" customWidth="1"/>
+    <col min="4" max="4" width="30.6328125" style="8" customWidth="1"/>
+    <col min="5" max="5" width="19.54296875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="35" style="8" customWidth="1"/>
+    <col min="7" max="7" width="17.26953125" style="8" customWidth="1"/>
+    <col min="8" max="16384" width="8.7265625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="C1" s="5" t="s">
+      <c r="B1" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="1">
+      <c r="C2" s="1">
+        <v>918</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" s="1">
         <v>12345</v>
       </c>
-      <c r="E2" s="1">
-        <v>830</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>40</v>
+      <c r="F2" s="19" t="s">
+        <v>39</v>
       </c>
       <c r="G2" s="1">
         <v>12345</v>
       </c>
-      <c r="H2" s="1">
-        <v>872</v>
-      </c>
-      <c r="I2" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="J2" s="1">
-        <v>12345</v>
-      </c>
-      <c r="K2" s="1">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="9"/>
       <c r="B3" s="1">
         <v>2</v>
       </c>
       <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="G3" s="1">
+      <c r="D3" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" s="1">
         <v>12345</v>
       </c>
-      <c r="H3" s="1">
-        <v>872</v>
-      </c>
-      <c r="I3" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="J3" s="1">
-        <v>12345</v>
-      </c>
-      <c r="K3" s="1">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="F3" s="19"/>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="9"/>
       <c r="B4" s="1">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="1">
-        <v>12345</v>
-      </c>
-      <c r="E4" s="1">
-        <v>831</v>
-      </c>
-      <c r="F4" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="G4" s="1">
-        <v>12345</v>
-      </c>
-      <c r="H4" s="1">
-        <v>873</v>
-      </c>
-      <c r="I4" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="J4" s="1">
-        <v>12345</v>
-      </c>
-      <c r="K4" s="1">
-        <v>873</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C4" s="1"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="9"/>
       <c r="B5" s="1">
         <v>4</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="1">
-        <v>12345</v>
-      </c>
-      <c r="E5" s="1">
-        <v>832</v>
-      </c>
-      <c r="F5" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="G5" s="1">
-        <v>12345</v>
-      </c>
-      <c r="H5" s="1">
-        <v>874</v>
-      </c>
-      <c r="I5" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="J5" s="1">
-        <v>12345</v>
-      </c>
-      <c r="K5" s="1">
-        <v>874</v>
-      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="F3" r:id="rId1" xr:uid="{D6323319-3F75-49A5-9F15-EF38138D42B0}"/>
-    <hyperlink ref="I3" r:id="rId2" xr:uid="{FCD8BB58-86CE-41E3-97AC-B55E5F8271F4}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
TC_004 TS_001 Script update v2
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6545B097-5AD4-43EC-A7EC-084ED1A1A216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E664E491-EF09-4346-BE9E-E284675F6145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="720" windowWidth="17610" windowHeight="8570" tabRatio="902" activeTab="4" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="4" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
   <sheets>
     <sheet name="BrowserSetup" sheetId="3" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="67">
   <si>
     <t>Username</t>
   </si>
@@ -214,13 +214,22 @@
     <t>Shyamal Kumar Mondal</t>
   </si>
   <si>
-    <t>Test Automation SOF</t>
-  </si>
-  <si>
     <t>TripId</t>
   </si>
   <si>
     <t>BudgetHolderUsername</t>
+  </si>
+  <si>
+    <t>Test Automation SOF 1</t>
+  </si>
+  <si>
+    <t>Test Automation SOF 2</t>
+  </si>
+  <si>
+    <t>1-Nov-2027 03:04:00 pm</t>
+  </si>
+  <si>
+    <t>1-Dec-2028 12:01:00 pm</t>
   </si>
 </sst>
 </file>
@@ -250,7 +259,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -284,6 +293,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -412,8 +427,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1003,7 +1020,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC28C683-2DE1-4543-8063-C85149D9A2B2}">
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:V8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.81640625" style="10" customWidth="1"/>
@@ -1142,7 +1159,7 @@
         <v>36</v>
       </c>
       <c r="R2" s="9" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="S2" s="9" t="s">
         <v>24</v>
@@ -1242,58 +1259,127 @@
       <c r="V5" s="9"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="9"/>
-      <c r="B6" s="9">
+      <c r="A6" s="26"/>
+      <c r="B6" s="26">
         <v>5</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="9"/>
-      <c r="Q6" s="9"/>
-      <c r="R6" s="9"/>
-      <c r="S6" s="9"/>
-      <c r="T6" s="9"/>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="C6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="26"/>
+      <c r="M6" s="26"/>
+      <c r="N6" s="26"/>
+      <c r="O6" s="26"/>
+      <c r="P6" s="26"/>
+      <c r="Q6" s="26"/>
+      <c r="R6" s="26"/>
+      <c r="S6" s="26"/>
+      <c r="T6" s="26"/>
+      <c r="U6" s="26"/>
+      <c r="V6" s="26"/>
+    </row>
+    <row r="7" spans="1:22" ht="116" x14ac:dyDescent="0.35">
       <c r="A7" s="9"/>
       <c r="B7" s="9">
         <v>6</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="9"/>
-      <c r="Q7" s="9"/>
-      <c r="R7" s="9"/>
-      <c r="S7" s="9"/>
-      <c r="T7" s="9"/>
-      <c r="U7" s="9"/>
-      <c r="V7" s="9"/>
+      <c r="C7" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="9">
+        <v>12345</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="L7" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="M7" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="N7" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="O7" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P7" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q7" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="R7" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="S7" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="T7" s="9">
+        <v>50</v>
+      </c>
+      <c r="U7" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="V7" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" ht="145" x14ac:dyDescent="0.35">
+      <c r="A8" s="9"/>
+      <c r="B8" s="9">
+        <v>7</v>
+      </c>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="9"/>
+      <c r="P8" s="9"/>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="9"/>
+      <c r="S8" s="9"/>
+      <c r="T8" s="9"/>
+      <c r="U8" s="9"/>
+      <c r="V8" s="9"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1319,11 +1405,11 @@
       <c r="B1" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>63</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>42</v>
@@ -1343,7 +1429,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>918</v>
+        <v>921</v>
       </c>
       <c r="D2" s="19" t="s">
         <v>38</v>
@@ -1364,7 +1450,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="1"/>
-      <c r="D3" s="25" t="s">
+      <c r="D3" t="s">
         <v>55</v>
       </c>
       <c r="E3" s="1">

</xml_diff>

<commit_message>
TC_004 TS_002 is done
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E664E491-EF09-4346-BE9E-E284675F6145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99CEE2F0-2CEC-4394-9EEC-B9A790BB60A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="4" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="71">
   <si>
     <t>Username</t>
   </si>
@@ -230,6 +230,18 @@
   </si>
   <si>
     <t>1-Dec-2028 12:01:00 pm</t>
+  </si>
+  <si>
+    <t>SupervisorReason</t>
+  </si>
+  <si>
+    <t>BudgetHolderReason</t>
+  </si>
+  <si>
+    <t>Test S</t>
+  </si>
+  <si>
+    <t>Test B</t>
   </si>
 </sst>
 </file>
@@ -1386,19 +1398,20 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B1CFC64-F19E-4BC4-A1E5-2FDFF8A8F1BB}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.7265625" style="10" customWidth="1"/>
-    <col min="2" max="3" width="10.7265625" style="8" customWidth="1"/>
-    <col min="4" max="4" width="30.6328125" style="8" customWidth="1"/>
-    <col min="5" max="5" width="19.54296875" style="8" customWidth="1"/>
-    <col min="6" max="6" width="35" style="8" customWidth="1"/>
-    <col min="7" max="7" width="17.26953125" style="8" customWidth="1"/>
-    <col min="8" max="16384" width="8.7265625" style="8"/>
+    <col min="2" max="4" width="10.7265625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="30.6328125" style="8" customWidth="1"/>
+    <col min="6" max="6" width="19.54296875" style="8" customWidth="1"/>
+    <col min="7" max="7" width="13.7265625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="35" style="8" customWidth="1"/>
+    <col min="9" max="9" width="17.26953125" style="8" customWidth="1"/>
+    <col min="10" max="16384" width="8.7265625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="21" t="s">
         <v>4</v>
       </c>
@@ -1408,20 +1421,26 @@
       <c r="C1" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>54</v>
       </c>
@@ -1429,57 +1448,69 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>921</v>
-      </c>
-      <c r="D2" s="19" t="s">
+        <v>927</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="E2" s="1">
+      <c r="F2" s="1">
         <v>12345</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="G2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H2" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="G2" s="1">
+      <c r="I2" s="1">
         <v>12345</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="9"/>
       <c r="B3" s="1">
         <v>2</v>
       </c>
       <c r="C3" s="1"/>
-      <c r="D3" t="s">
+      <c r="D3" s="1"/>
+      <c r="E3" t="s">
         <v>55</v>
       </c>
-      <c r="E3" s="1">
+      <c r="F3" s="1">
         <v>12345</v>
       </c>
-      <c r="F3" s="19"/>
       <c r="G3" s="1"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H3" s="19"/>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="9"/>
       <c r="B4" s="1">
         <v>3</v>
       </c>
       <c r="C4" s="1"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="19"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H4" s="19"/>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="9"/>
       <c r="B5" s="1">
         <v>4</v>
       </c>
       <c r="C5" s="1"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="19"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="1"/>
       <c r="G5" s="1"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
TC_004 TS_003 is done
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99CEE2F0-2CEC-4394-9EEC-B9A790BB60A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5AD6569-30BE-44CA-A6A3-A0B84B2451AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="4" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="70">
   <si>
     <t>Username</t>
   </si>
@@ -239,9 +239,6 @@
   </si>
   <si>
     <t>Test S</t>
-  </si>
-  <si>
-    <t>Test B</t>
   </si>
 </sst>
 </file>
@@ -1448,11 +1445,9 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>927</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>70</v>
-      </c>
+        <v>928</v>
+      </c>
+      <c r="D2" s="1"/>
       <c r="E2" s="19" t="s">
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
TC_004 TS_004 is done
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5AD6569-30BE-44CA-A6A3-A0B84B2451AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E878D67-AF71-4E05-AAAB-18EA7626DFFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="4" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
@@ -1445,7 +1445,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>928</v>
+        <v>933</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="19" t="s">

</xml_diff>

<commit_message>
TC_004 TS_005 is done.
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E878D67-AF71-4E05-AAAB-18EA7626DFFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEB95524-C786-4E57-AF93-2FE52DEB4DD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="4" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="71">
   <si>
     <t>Username</t>
   </si>
@@ -239,6 +239,9 @@
   </si>
   <si>
     <t>Test S</t>
+  </si>
+  <si>
+    <t>Test B</t>
   </si>
 </sst>
 </file>
@@ -1445,7 +1448,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>933</v>
+        <v>935</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="19" t="s">
@@ -1470,7 +1473,9 @@
         <v>2</v>
       </c>
       <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
+      <c r="D3" s="1" t="s">
+        <v>70</v>
+      </c>
       <c r="E3" t="s">
         <v>55</v>
       </c>

</xml_diff>

<commit_message>
TC_005 is in progress
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BDB0B00-16E8-4BA0-B179-F2CC2D1F3489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52FBF367-B9A7-4E06-BCB2-DAF754BF391D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="4" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="5" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
   <sheets>
     <sheet name="BrowserSetup" sheetId="3" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="LogoutData" sheetId="2" r:id="rId3"/>
     <sheet name="TripRequestData" sheetId="4" r:id="rId4"/>
     <sheet name="TripApprovalData" sheetId="7" r:id="rId5"/>
+    <sheet name="SOFData" sheetId="9" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="100">
   <si>
     <t>Username</t>
   </si>
@@ -242,6 +243,93 @@
   </si>
   <si>
     <t>Test B</t>
+  </si>
+  <si>
+    <t>TestSOF-1</t>
+  </si>
+  <si>
+    <t>Narrative</t>
+  </si>
+  <si>
+    <t>Account Code</t>
+  </si>
+  <si>
+    <t>Cost Center</t>
+  </si>
+  <si>
+    <t>Project</t>
+  </si>
+  <si>
+    <t>SOF</t>
+  </si>
+  <si>
+    <t>DRC</t>
+  </si>
+  <si>
+    <t>Activity</t>
+  </si>
+  <si>
+    <t>Budget Holder</t>
+  </si>
+  <si>
+    <t>Percentage</t>
+  </si>
+  <si>
+    <t>SOF Name</t>
+  </si>
+  <si>
+    <t>TestSOF-2</t>
+  </si>
+  <si>
+    <t>TS-1</t>
+  </si>
+  <si>
+    <t>TS-2</t>
+  </si>
+  <si>
+    <t>05000A</t>
+  </si>
+  <si>
+    <t>05000B</t>
+  </si>
+  <si>
+    <t>0501000</t>
+  </si>
+  <si>
+    <t>0501019</t>
+  </si>
+  <si>
+    <t>20801026</t>
+  </si>
+  <si>
+    <t>208010260054</t>
+  </si>
+  <si>
+    <t>AC04A</t>
+  </si>
+  <si>
+    <t>Mohi Uddin</t>
+  </si>
+  <si>
+    <t>70</t>
+  </si>
+  <si>
+    <t>Test-1</t>
+  </si>
+  <si>
+    <t>84002731</t>
+  </si>
+  <si>
+    <t>840027310002</t>
+  </si>
+  <si>
+    <t>PM08A</t>
+  </si>
+  <si>
+    <t>Rokybul Imrose</t>
+  </si>
+  <si>
+    <t>30</t>
   </si>
 </sst>
 </file>
@@ -271,7 +359,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -310,7 +398,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -367,7 +461,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -443,6 +537,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1271,30 +1368,30 @@
       <c r="V5" s="9"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="26"/>
-      <c r="B6" s="26">
+      <c r="A6" s="27"/>
+      <c r="B6" s="27">
         <v>5</v>
       </c>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26"/>
-      <c r="J6" s="26"/>
-      <c r="K6" s="26"/>
-      <c r="L6" s="26"/>
-      <c r="M6" s="26"/>
-      <c r="N6" s="26"/>
-      <c r="O6" s="26"/>
-      <c r="P6" s="26"/>
-      <c r="Q6" s="26"/>
-      <c r="R6" s="26"/>
-      <c r="S6" s="26"/>
-      <c r="T6" s="26"/>
-      <c r="U6" s="26"/>
-      <c r="V6" s="26"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="27"/>
+      <c r="K6" s="27"/>
+      <c r="L6" s="27"/>
+      <c r="M6" s="27"/>
+      <c r="N6" s="27"/>
+      <c r="O6" s="27"/>
+      <c r="P6" s="27"/>
+      <c r="Q6" s="27"/>
+      <c r="R6" s="27"/>
+      <c r="S6" s="27"/>
+      <c r="T6" s="27"/>
+      <c r="U6" s="27"/>
+      <c r="V6" s="27"/>
     </row>
     <row r="7" spans="1:22" ht="116" x14ac:dyDescent="0.35">
       <c r="A7" s="9"/>
@@ -1517,4 +1614,262 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19F63B13-47E9-468A-80A4-B58BA6E90505}">
+  <dimension ref="A1:N9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="9.36328125" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7265625" style="10"/>
+    <col min="3" max="3" width="18.81640625" style="10" customWidth="1"/>
+    <col min="4" max="4" width="16.6328125" style="10" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" style="10" customWidth="1"/>
+    <col min="6" max="6" width="10.7265625" style="10" customWidth="1"/>
+    <col min="7" max="7" width="10.90625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="10.7265625" style="10" customWidth="1"/>
+    <col min="9" max="9" width="10.90625" style="10" customWidth="1"/>
+    <col min="10" max="11" width="11" style="10" customWidth="1"/>
+    <col min="12" max="12" width="10.08984375" style="10" customWidth="1"/>
+    <col min="13" max="13" width="11.08984375" style="10" customWidth="1"/>
+    <col min="14" max="16384" width="8.7265625" style="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="G1" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="H1" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="I1" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="J1" s="26" t="s">
+        <v>77</v>
+      </c>
+      <c r="K1" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="L1" s="26" t="s">
+        <v>79</v>
+      </c>
+      <c r="M1" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="N1" s="26" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="9">
+        <v>1</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="9">
+        <v>12345</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="K2" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="L2" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="M2" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="N2" s="9" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9">
+        <v>2</v>
+      </c>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="M3" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="N3" s="9"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" s="27"/>
+      <c r="B4" s="27">
+        <v>3</v>
+      </c>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
+      <c r="M4" s="27"/>
+      <c r="N4" s="27"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5" s="9"/>
+      <c r="B5" s="9">
+        <v>4</v>
+      </c>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9">
+        <v>5</v>
+      </c>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A7" s="9"/>
+      <c r="B7" s="9">
+        <v>6</v>
+      </c>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A8" s="9"/>
+      <c r="B8" s="9">
+        <v>7</v>
+      </c>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A9" s="9"/>
+      <c r="B9" s="9">
+        <v>8</v>
+      </c>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
TC_005 TS_001 is done
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52FBF367-B9A7-4E06-BCB2-DAF754BF391D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E55A99B-AA08-4E28-8AF0-B9DC4D2D6A56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="5" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
+    <workbookView xWindow="720" yWindow="720" windowWidth="17610" windowHeight="8570" tabRatio="902" activeTab="5" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
   <sheets>
     <sheet name="BrowserSetup" sheetId="3" r:id="rId1"/>
@@ -251,12 +251,6 @@
     <t>Narrative</t>
   </si>
   <si>
-    <t>Account Code</t>
-  </si>
-  <si>
-    <t>Cost Center</t>
-  </si>
-  <si>
     <t>Project</t>
   </si>
   <si>
@@ -269,15 +263,9 @@
     <t>Activity</t>
   </si>
   <si>
-    <t>Budget Holder</t>
-  </si>
-  <si>
     <t>Percentage</t>
   </si>
   <si>
-    <t>SOF Name</t>
-  </si>
-  <si>
     <t>TestSOF-2</t>
   </si>
   <si>
@@ -287,49 +275,61 @@
     <t>TS-2</t>
   </si>
   <si>
+    <t>Mohi Uddin</t>
+  </si>
+  <si>
+    <t>70</t>
+  </si>
+  <si>
+    <t>Test-1</t>
+  </si>
+  <si>
+    <t>Rokybul Imrose</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>AccountCode</t>
+  </si>
+  <si>
+    <t>CostCenter</t>
+  </si>
+  <si>
+    <t>BudgetHolder</t>
+  </si>
+  <si>
+    <t>SOFName</t>
+  </si>
+  <si>
+    <t>BGD-cf-17 - Integrated education and child protection services for vulnerable Rohingya refugee children in Cox’s Bazar - 2022</t>
+  </si>
+  <si>
+    <t>BGD_Danida SPA 2023-2025 Lot HUM</t>
+  </si>
+  <si>
+    <t>BG4AGYO054BG-2.1.1 Sr. Programme Manager-CP-(1)-(15%)</t>
+  </si>
+  <si>
+    <t>Advocacy/Campaign Event</t>
+  </si>
+  <si>
+    <t>BGD - Cholo Shikhi Khelar Chholey (CSKC) - 2015 [MDM]</t>
+  </si>
+  <si>
+    <t>BGD_ PVH Hyper Designated Contribution</t>
+  </si>
+  <si>
+    <t>202-BGD Employee Engagement and Communications</t>
+  </si>
+  <si>
+    <t>SCI Centre_HR planning</t>
+  </si>
+  <si>
     <t>05000A</t>
   </si>
   <si>
     <t>05000B</t>
-  </si>
-  <si>
-    <t>0501000</t>
-  </si>
-  <si>
-    <t>0501019</t>
-  </si>
-  <si>
-    <t>20801026</t>
-  </si>
-  <si>
-    <t>208010260054</t>
-  </si>
-  <si>
-    <t>AC04A</t>
-  </si>
-  <si>
-    <t>Mohi Uddin</t>
-  </si>
-  <si>
-    <t>70</t>
-  </si>
-  <si>
-    <t>Test-1</t>
-  </si>
-  <si>
-    <t>84002731</t>
-  </si>
-  <si>
-    <t>840027310002</t>
-  </si>
-  <si>
-    <t>PM08A</t>
-  </si>
-  <si>
-    <t>Rokybul Imrose</t>
-  </si>
-  <si>
-    <t>30</t>
   </si>
 </sst>
 </file>
@@ -1626,14 +1626,15 @@
     <col min="3" max="3" width="18.81640625" style="10" customWidth="1"/>
     <col min="4" max="4" width="16.6328125" style="10" customWidth="1"/>
     <col min="5" max="5" width="11.54296875" style="10" customWidth="1"/>
-    <col min="6" max="6" width="10.7265625" style="10" customWidth="1"/>
+    <col min="6" max="6" width="11.6328125" style="10" customWidth="1"/>
     <col min="7" max="7" width="10.90625" style="10" customWidth="1"/>
     <col min="8" max="8" width="10.7265625" style="10" customWidth="1"/>
     <col min="9" max="9" width="10.90625" style="10" customWidth="1"/>
     <col min="10" max="11" width="11" style="10" customWidth="1"/>
     <col min="12" max="12" width="10.08984375" style="10" customWidth="1"/>
     <col min="13" max="13" width="11.08984375" style="10" customWidth="1"/>
-    <col min="14" max="16384" width="8.7265625" style="10"/>
+    <col min="14" max="14" width="10.90625" style="10" customWidth="1"/>
+    <col min="15" max="16384" width="8.7265625" style="10"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="29" x14ac:dyDescent="0.35">
@@ -1653,34 +1654,34 @@
         <v>72</v>
       </c>
       <c r="F1" s="26" t="s">
+        <v>86</v>
+      </c>
+      <c r="G1" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="H1" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="G1" s="26" t="s">
+      <c r="I1" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="H1" s="26" t="s">
+      <c r="J1" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="I1" s="26" t="s">
+      <c r="K1" s="26" t="s">
         <v>76</v>
       </c>
-      <c r="J1" s="26" t="s">
+      <c r="L1" s="26" t="s">
+        <v>88</v>
+      </c>
+      <c r="M1" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="K1" s="26" t="s">
-        <v>78</v>
-      </c>
-      <c r="L1" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="M1" s="26" t="s">
-        <v>80</v>
-      </c>
       <c r="N1" s="26" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="174" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>54</v>
       </c>
@@ -1697,34 +1698,34 @@
         <v>71</v>
       </c>
       <c r="F2" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="K2" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="L2" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="M2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="N2" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="G2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="J2" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="K2" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="L2" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="M2" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="N2" s="9" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:14" ht="87" x14ac:dyDescent="0.35">
       <c r="A3" s="9"/>
       <c r="B3" s="9">
         <v>2</v>
@@ -1732,16 +1733,16 @@
       <c r="C3" s="9"/>
       <c r="D3" s="9"/>
       <c r="E3" s="9" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="I3" s="9" t="s">
         <v>95</v>
@@ -1753,10 +1754,10 @@
         <v>97</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="N3" s="9"/>
     </row>

</xml_diff>

<commit_message>
TC_005 TS_002 is done
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E55A99B-AA08-4E28-8AF0-B9DC4D2D6A56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0578736E-A10B-4D8B-BF6A-5B2C55C64B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="720" windowWidth="17610" windowHeight="8570" tabRatio="902" activeTab="5" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="5" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
   <sheets>
     <sheet name="BrowserSetup" sheetId="3" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="102">
   <si>
     <t>Username</t>
   </si>
@@ -330,6 +330,12 @@
   </si>
   <si>
     <t>05000B</t>
+  </si>
+  <si>
+    <t>SOFNameForDeletion</t>
+  </si>
+  <si>
+    <t>SOFNameForEdit</t>
   </si>
 </sst>
 </file>
@@ -1618,7 +1624,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19F63B13-47E9-468A-80A4-B58BA6E90505}">
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.36328125" style="10" bestFit="1" customWidth="1"/>
@@ -1634,10 +1640,12 @@
     <col min="12" max="12" width="10.08984375" style="10" customWidth="1"/>
     <col min="13" max="13" width="11.08984375" style="10" customWidth="1"/>
     <col min="14" max="14" width="10.90625" style="10" customWidth="1"/>
-    <col min="15" max="16384" width="8.7265625" style="10"/>
+    <col min="15" max="15" width="12" style="10" customWidth="1"/>
+    <col min="16" max="16" width="9.7265625" style="10" customWidth="1"/>
+    <col min="17" max="16384" width="8.7265625" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="22" t="s">
         <v>4</v>
       </c>
@@ -1680,8 +1688,14 @@
       <c r="N1" s="26" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" ht="174" x14ac:dyDescent="0.35">
+      <c r="O1" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="P1" s="26" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="174" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>54</v>
       </c>
@@ -1724,8 +1738,14 @@
       <c r="N2" s="9" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" ht="87" x14ac:dyDescent="0.35">
+      <c r="O2" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="P2" s="9" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="87" x14ac:dyDescent="0.35">
       <c r="A3" s="9"/>
       <c r="B3" s="9">
         <v>2</v>
@@ -1760,8 +1780,10 @@
         <v>85</v>
       </c>
       <c r="N3" s="9"/>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="27"/>
       <c r="B4" s="27">
         <v>3</v>
@@ -1778,8 +1800,10 @@
       <c r="L4" s="27"/>
       <c r="M4" s="27"/>
       <c r="N4" s="27"/>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="9"/>
       <c r="B5" s="9">
         <v>4</v>
@@ -1796,8 +1820,10 @@
       <c r="L5" s="9"/>
       <c r="M5" s="9"/>
       <c r="N5" s="9"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O5" s="9"/>
+      <c r="P5" s="9"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="9"/>
       <c r="B6" s="9">
         <v>5</v>
@@ -1814,8 +1840,10 @@
       <c r="L6" s="9"/>
       <c r="M6" s="9"/>
       <c r="N6" s="9"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O6" s="9"/>
+      <c r="P6" s="9"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="9"/>
       <c r="B7" s="9">
         <v>6</v>
@@ -1832,8 +1860,10 @@
       <c r="L7" s="9"/>
       <c r="M7" s="9"/>
       <c r="N7" s="9"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O7" s="9"/>
+      <c r="P7" s="9"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="9"/>
       <c r="B8" s="9">
         <v>7</v>
@@ -1850,8 +1880,10 @@
       <c r="L8" s="9"/>
       <c r="M8" s="9"/>
       <c r="N8" s="9"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O8" s="9"/>
+      <c r="P8" s="9"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="9"/>
       <c r="B9" s="9">
         <v>8</v>
@@ -1868,6 +1900,8 @@
       <c r="L9" s="9"/>
       <c r="M9" s="9"/>
       <c r="N9" s="9"/>
+      <c r="O9" s="9"/>
+      <c r="P9" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
TC_004 is in progress and TC_005 Script updated
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,17 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0578736E-A10B-4D8B-BF6A-5B2C55C64B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C4B41B8-9157-4F3E-9588-DD26EE062DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" activeTab="5" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
+    <workbookView xWindow="720" yWindow="720" windowWidth="17610" windowHeight="8570" tabRatio="902" firstSheet="5" activeTab="6" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
   <sheets>
     <sheet name="BrowserSetup" sheetId="3" r:id="rId1"/>
     <sheet name="LoginData" sheetId="1" r:id="rId2"/>
     <sheet name="LogoutData" sheetId="2" r:id="rId3"/>
     <sheet name="TripRequestData" sheetId="4" r:id="rId4"/>
-    <sheet name="TripApprovalData" sheetId="7" r:id="rId5"/>
-    <sheet name="SOFData" sheetId="9" r:id="rId6"/>
+    <sheet name="TripApprovalData_TS_001" sheetId="7" r:id="rId5"/>
+    <sheet name="TripApprovalData_TS_002" sheetId="10" r:id="rId6"/>
+    <sheet name="TripApprovalData_TS_003" sheetId="11" r:id="rId7"/>
+    <sheet name="TripApprovalData_TS_004" sheetId="12" r:id="rId8"/>
+    <sheet name="TripApprovalData_TS_005" sheetId="13" r:id="rId9"/>
+    <sheet name="TripApprovalData_TS_006" sheetId="14" r:id="rId10"/>
+    <sheet name="SOFData" sheetId="9" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="101">
   <si>
     <t>Username</t>
   </si>
@@ -281,9 +286,6 @@
     <t>70</t>
   </si>
   <si>
-    <t>Test-1</t>
-  </si>
-  <si>
     <t>Rokybul Imrose</t>
   </si>
   <si>
@@ -335,7 +337,7 @@
     <t>SOFNameForDeletion</t>
   </si>
   <si>
-    <t>SOFNameForEdit</t>
+    <t>Test-2</t>
   </si>
 </sst>
 </file>
@@ -365,7 +367,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -414,8 +416,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF66"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -462,12 +476,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -480,9 +507,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -527,9 +551,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -539,15 +560,30 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -555,6 +591,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFFF66"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -889,15 +930,15 @@
     <col min="1" max="1" width="11.6328125" style="2" customWidth="1"/>
     <col min="2" max="2" width="7.54296875" style="2" customWidth="1"/>
     <col min="3" max="3" width="15.26953125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="57.26953125" style="13" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="13"/>
+    <col min="4" max="4" width="57.26953125" style="12" customWidth="1"/>
+    <col min="5" max="16384" width="8.7265625" style="12"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="16" t="s">
         <v>51</v>
       </c>
       <c r="C1" s="4" t="s">
@@ -917,7 +958,7 @@
       <c r="C2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="13" t="s">
         <v>50</v>
       </c>
     </row>
@@ -929,7 +970,7 @@
       <c r="C3" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="13" t="s">
         <v>3</v>
       </c>
     </row>
@@ -941,7 +982,7 @@
       <c r="C4" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="13" t="s">
         <v>50</v>
       </c>
     </row>
@@ -953,7 +994,7 @@
       <c r="C5" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="13" t="s">
         <v>3</v>
       </c>
     </row>
@@ -963,7 +1004,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="3"/>
-      <c r="D6" s="14"/>
+      <c r="D6" s="13"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
@@ -971,7 +1012,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="14"/>
+      <c r="D7" s="13"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -980,6 +1021,573 @@
     <hyperlink ref="D2" r:id="rId3" xr:uid="{9E2AC4D9-B9A1-4BA6-9745-5A8541B67764}"/>
     <hyperlink ref="D4" r:id="rId4" xr:uid="{1E21B194-8990-438C-B182-42930FDCE507}"/>
   </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9611332-2F90-450D-9C67-DA6920B878FA}">
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.7265625" style="9" customWidth="1"/>
+    <col min="2" max="4" width="10.7265625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="30.6328125" style="7" customWidth="1"/>
+    <col min="6" max="6" width="19.54296875" style="7" customWidth="1"/>
+    <col min="7" max="7" width="13.7265625" style="7" customWidth="1"/>
+    <col min="8" max="8" width="35" style="7" customWidth="1"/>
+    <col min="9" max="9" width="17.26953125" style="7" customWidth="1"/>
+    <col min="10" max="16384" width="8.7265625" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="H1" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="I1" s="26" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="29">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1">
+        <v>951</v>
+      </c>
+      <c r="D2" s="1"/>
+      <c r="E2" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="1">
+        <v>12345</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="1">
+        <v>12345</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="8"/>
+      <c r="B3" s="29">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="1">
+        <v>12345</v>
+      </c>
+      <c r="G3" s="1"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="28"/>
+      <c r="B4" s="29">
+        <v>3</v>
+      </c>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="29"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="28"/>
+      <c r="B5" s="29">
+        <v>4</v>
+      </c>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="29"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="28"/>
+      <c r="B6" s="29">
+        <v>5</v>
+      </c>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="29"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="28"/>
+      <c r="B7" s="29">
+        <v>6</v>
+      </c>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="29"/>
+      <c r="H7" s="29"/>
+      <c r="I7" s="29"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="28"/>
+      <c r="B8" s="29">
+        <v>7</v>
+      </c>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="29"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="28"/>
+      <c r="B9" s="29">
+        <v>8</v>
+      </c>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="29"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="28"/>
+      <c r="B10" s="29">
+        <v>9</v>
+      </c>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="28"/>
+      <c r="B11" s="29">
+        <v>10</v>
+      </c>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="29"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="28"/>
+      <c r="B12" s="29">
+        <v>11</v>
+      </c>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="29"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" s="28"/>
+      <c r="B13" s="29">
+        <v>12</v>
+      </c>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" s="28"/>
+      <c r="B14" s="29">
+        <v>13</v>
+      </c>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="29"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="28"/>
+      <c r="B15" s="29">
+        <v>14</v>
+      </c>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="29"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="28"/>
+      <c r="B16" s="29">
+        <v>15</v>
+      </c>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="29"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" s="28"/>
+      <c r="B17" s="29">
+        <v>16</v>
+      </c>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="29"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" s="28"/>
+      <c r="B18" s="29">
+        <v>17</v>
+      </c>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="29"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{73831D83-4816-412C-B6DE-323CD2B07E76}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19F63B13-47E9-468A-80A4-B58BA6E90505}">
+  <dimension ref="A1:O9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="9.36328125" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7265625" style="9"/>
+    <col min="3" max="3" width="18.81640625" style="9" customWidth="1"/>
+    <col min="4" max="4" width="16.6328125" style="9" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" style="9" customWidth="1"/>
+    <col min="6" max="6" width="11.6328125" style="9" customWidth="1"/>
+    <col min="7" max="7" width="10.90625" style="9" customWidth="1"/>
+    <col min="8" max="8" width="10.7265625" style="9" customWidth="1"/>
+    <col min="9" max="9" width="10.90625" style="9" customWidth="1"/>
+    <col min="10" max="11" width="11" style="9" customWidth="1"/>
+    <col min="12" max="12" width="10.08984375" style="9" customWidth="1"/>
+    <col min="13" max="13" width="11.08984375" style="9" customWidth="1"/>
+    <col min="14" max="14" width="10.90625" style="9" customWidth="1"/>
+    <col min="15" max="15" width="12" style="9" customWidth="1"/>
+    <col min="16" max="16384" width="8.7265625" style="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="23" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="G1" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="H1" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="I1" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="J1" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="K1" s="23" t="s">
+        <v>76</v>
+      </c>
+      <c r="L1" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="M1" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="N1" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="O1" s="23" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="174" x14ac:dyDescent="0.35">
+      <c r="A2" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="8">
+        <v>1</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="8">
+        <v>12345</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="M2" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="N2" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="87" x14ac:dyDescent="0.35">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8">
+        <v>2</v>
+      </c>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A4" s="24"/>
+      <c r="B4" s="24">
+        <v>3</v>
+      </c>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A5" s="8"/>
+      <c r="B5" s="8">
+        <v>4</v>
+      </c>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8">
+        <v>5</v>
+      </c>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8">
+        <v>6</v>
+      </c>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8">
+        <v>7</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A9" s="8"/>
+      <c r="B9" s="8">
+        <v>8</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -999,10 +1607,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="16" t="s">
         <v>51</v>
       </c>
       <c r="C1" s="4" t="s">
@@ -1014,7 +1622,7 @@
       <c r="E1" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="11" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1034,7 +1642,7 @@
       <c r="E2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="14" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1046,7 +1654,7 @@
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
-      <c r="F3" s="16"/>
+      <c r="F3" s="15"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="3"/>
@@ -1056,7 +1664,7 @@
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
-      <c r="F4" s="16"/>
+      <c r="F4" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1077,16 +1685,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="17" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1138,360 +1746,360 @@
   <dimension ref="A1:V8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.81640625" style="10" customWidth="1"/>
-    <col min="2" max="2" width="5.6328125" style="10" customWidth="1"/>
-    <col min="3" max="4" width="8.7265625" style="10"/>
-    <col min="5" max="5" width="13.36328125" style="10" customWidth="1"/>
-    <col min="6" max="7" width="15.36328125" style="10" customWidth="1"/>
-    <col min="8" max="9" width="8.7265625" style="10"/>
-    <col min="10" max="10" width="15.08984375" style="10" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.08984375" style="10" customWidth="1"/>
-    <col min="12" max="12" width="8.7265625" style="10"/>
-    <col min="13" max="13" width="10.81640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="14" max="16" width="8.7265625" style="10"/>
-    <col min="17" max="17" width="10.81640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="8.7265625" style="10"/>
+    <col min="1" max="1" width="11.81640625" style="9" customWidth="1"/>
+    <col min="2" max="2" width="5.6328125" style="9" customWidth="1"/>
+    <col min="3" max="4" width="8.7265625" style="9"/>
+    <col min="5" max="5" width="13.36328125" style="9" customWidth="1"/>
+    <col min="6" max="7" width="15.36328125" style="9" customWidth="1"/>
+    <col min="8" max="9" width="8.7265625" style="9"/>
+    <col min="10" max="10" width="15.08984375" style="9" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.08984375" style="9" customWidth="1"/>
+    <col min="12" max="12" width="8.7265625" style="9"/>
+    <col min="13" max="13" width="10.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="8.7265625" style="9"/>
+    <col min="17" max="17" width="10.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="8.7265625" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="L1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="M1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="N1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="O1" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="P1" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="Q1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="R1" s="7" t="s">
+      <c r="R1" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="S1" s="7" t="s">
+      <c r="S1" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="T1" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="U1" s="7" t="s">
+      <c r="U1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="V1" s="7" t="s">
+      <c r="V1" s="6" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="116" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="8">
         <v>1</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="8">
         <v>12345</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="K2" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="L2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="M2" s="24" t="s">
+      <c r="M2" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="N2" s="9" t="s">
+      <c r="N2" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="O2" s="9" t="s">
+      <c r="O2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="P2" s="9" t="s">
+      <c r="P2" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="Q2" s="24" t="s">
+      <c r="Q2" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="R2" s="9" t="s">
+      <c r="R2" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="S2" s="9" t="s">
+      <c r="S2" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="T2" s="9">
+      <c r="T2" s="8">
         <v>50</v>
       </c>
-      <c r="U2" s="9" t="s">
+      <c r="U2" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="V2" s="9" t="s">
+      <c r="V2" s="8" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:22" ht="145" x14ac:dyDescent="0.35">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8">
         <v>2</v>
       </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9" t="s">
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
-      <c r="Q3" s="9"/>
-      <c r="R3" s="9"/>
-      <c r="S3" s="9"/>
-      <c r="T3" s="9"/>
-      <c r="U3" s="9"/>
-      <c r="V3" s="9"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="8"/>
+      <c r="R3" s="8"/>
+      <c r="S3" s="8"/>
+      <c r="T3" s="8"/>
+      <c r="U3" s="8"/>
+      <c r="V3" s="8"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A4" s="9"/>
-      <c r="B4" s="9">
+      <c r="A4" s="8"/>
+      <c r="B4" s="8">
         <v>3</v>
       </c>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9" t="s">
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="9"/>
-      <c r="Q4" s="9"/>
-      <c r="R4" s="9"/>
-      <c r="S4" s="9"/>
-      <c r="T4" s="9"/>
-      <c r="U4" s="9"/>
-      <c r="V4" s="9"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="8"/>
+      <c r="P4" s="8"/>
+      <c r="Q4" s="8"/>
+      <c r="R4" s="8"/>
+      <c r="S4" s="8"/>
+      <c r="T4" s="8"/>
+      <c r="U4" s="8"/>
+      <c r="V4" s="8"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A5" s="9"/>
-      <c r="B5" s="9">
+      <c r="A5" s="8"/>
+      <c r="B5" s="8">
         <v>4</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9" t="s">
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
-      <c r="N5" s="9"/>
-      <c r="O5" s="9"/>
-      <c r="P5" s="9"/>
-      <c r="Q5" s="9"/>
-      <c r="R5" s="9"/>
-      <c r="S5" s="9"/>
-      <c r="T5" s="9"/>
-      <c r="U5" s="9"/>
-      <c r="V5" s="9"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8"/>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="8"/>
+      <c r="R5" s="8"/>
+      <c r="S5" s="8"/>
+      <c r="T5" s="8"/>
+      <c r="U5" s="8"/>
+      <c r="V5" s="8"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="27"/>
-      <c r="B6" s="27">
+      <c r="A6" s="24"/>
+      <c r="B6" s="24">
         <v>5</v>
       </c>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
-      <c r="K6" s="27"/>
-      <c r="L6" s="27"/>
-      <c r="M6" s="27"/>
-      <c r="N6" s="27"/>
-      <c r="O6" s="27"/>
-      <c r="P6" s="27"/>
-      <c r="Q6" s="27"/>
-      <c r="R6" s="27"/>
-      <c r="S6" s="27"/>
-      <c r="T6" s="27"/>
-      <c r="U6" s="27"/>
-      <c r="V6" s="27"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="24"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="24"/>
+      <c r="M6" s="24"/>
+      <c r="N6" s="24"/>
+      <c r="O6" s="24"/>
+      <c r="P6" s="24"/>
+      <c r="Q6" s="24"/>
+      <c r="R6" s="24"/>
+      <c r="S6" s="24"/>
+      <c r="T6" s="24"/>
+      <c r="U6" s="24"/>
+      <c r="V6" s="24"/>
     </row>
     <row r="7" spans="1:22" ht="116" x14ac:dyDescent="0.35">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8">
         <v>6</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="8">
         <v>12345</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="I7" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="J7" s="9" t="s">
+      <c r="J7" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="K7" s="9" t="s">
+      <c r="K7" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="L7" s="9" t="s">
+      <c r="L7" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="M7" s="24" t="s">
+      <c r="M7" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="N7" s="9" t="s">
+      <c r="N7" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="O7" s="9" t="s">
+      <c r="O7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="P7" s="9" t="s">
+      <c r="P7" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="Q7" s="24" t="s">
+      <c r="Q7" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="R7" s="9" t="s">
+      <c r="R7" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="S7" s="9" t="s">
+      <c r="S7" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="T7" s="9">
+      <c r="T7" s="8">
         <v>50</v>
       </c>
-      <c r="U7" s="9" t="s">
+      <c r="U7" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="V7" s="9" t="s">
+      <c r="V7" s="8" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:22" ht="145" x14ac:dyDescent="0.35">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8">
         <v>7</v>
       </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9" t="s">
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
-      <c r="Q8" s="9"/>
-      <c r="R8" s="9"/>
-      <c r="S8" s="9"/>
-      <c r="T8" s="9"/>
-      <c r="U8" s="9"/>
-      <c r="V8" s="9"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="8"/>
+      <c r="T8" s="8"/>
+      <c r="U8" s="8"/>
+      <c r="V8" s="8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1501,24 +2109,24 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B1CFC64-F19E-4BC4-A1E5-2FDFF8A8F1BB}">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.7265625" style="10" customWidth="1"/>
-    <col min="2" max="4" width="10.7265625" style="8" customWidth="1"/>
-    <col min="5" max="5" width="30.6328125" style="8" customWidth="1"/>
-    <col min="6" max="6" width="19.54296875" style="8" customWidth="1"/>
-    <col min="7" max="7" width="13.7265625" style="8" customWidth="1"/>
-    <col min="8" max="8" width="35" style="8" customWidth="1"/>
-    <col min="9" max="9" width="17.26953125" style="8" customWidth="1"/>
-    <col min="10" max="16384" width="8.7265625" style="8"/>
+    <col min="1" max="1" width="10.7265625" style="9" customWidth="1"/>
+    <col min="2" max="4" width="10.7265625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="30.6328125" style="7" customWidth="1"/>
+    <col min="6" max="6" width="19.54296875" style="7" customWidth="1"/>
+    <col min="7" max="7" width="13.7265625" style="7" customWidth="1"/>
+    <col min="8" max="8" width="35" style="7" customWidth="1"/>
+    <col min="9" max="9" width="17.26953125" style="7" customWidth="1"/>
+    <col min="10" max="16384" width="8.7265625" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="19" t="s">
         <v>51</v>
       </c>
       <c r="C1" s="25" t="s">
@@ -1527,34 +2135,34 @@
       <c r="D1" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="26" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="29">
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>935</v>
+        <v>946</v>
       </c>
       <c r="D2" s="1"/>
-      <c r="E2" s="19" t="s">
+      <c r="E2" s="18" t="s">
         <v>38</v>
       </c>
       <c r="F2" s="1">
@@ -1563,7 +2171,7 @@
       <c r="G2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="18" t="s">
         <v>39</v>
       </c>
       <c r="I2" s="1">
@@ -1571,8 +2179,8 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="9"/>
-      <c r="B3" s="1">
+      <c r="A3" s="8"/>
+      <c r="B3" s="29">
         <v>2</v>
       </c>
       <c r="C3" s="1"/>
@@ -1586,34 +2194,203 @@
         <v>12345</v>
       </c>
       <c r="G3" s="1"/>
-      <c r="H3" s="19"/>
+      <c r="H3" s="18"/>
       <c r="I3" s="1"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="9"/>
-      <c r="B4" s="1">
+      <c r="A4" s="28"/>
+      <c r="B4" s="29">
         <v>3</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="1"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="29"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" s="9"/>
-      <c r="B5" s="1">
+      <c r="A5" s="28"/>
+      <c r="B5" s="29">
         <v>4</v>
       </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="1"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="29"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="28"/>
+      <c r="B6" s="29">
+        <v>5</v>
+      </c>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="29"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="28"/>
+      <c r="B7" s="29">
+        <v>6</v>
+      </c>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="29"/>
+      <c r="H7" s="29"/>
+      <c r="I7" s="29"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="28"/>
+      <c r="B8" s="29">
+        <v>7</v>
+      </c>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="29"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="28"/>
+      <c r="B9" s="29">
+        <v>8</v>
+      </c>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="29"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="28"/>
+      <c r="B10" s="29">
+        <v>9</v>
+      </c>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="28"/>
+      <c r="B11" s="29">
+        <v>10</v>
+      </c>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="29"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="28"/>
+      <c r="B12" s="29">
+        <v>11</v>
+      </c>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="29"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" s="28"/>
+      <c r="B13" s="29">
+        <v>12</v>
+      </c>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" s="28"/>
+      <c r="B14" s="29">
+        <v>13</v>
+      </c>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="29"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="28"/>
+      <c r="B15" s="29">
+        <v>14</v>
+      </c>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="29"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="28"/>
+      <c r="B16" s="29">
+        <v>15</v>
+      </c>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="29"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" s="28"/>
+      <c r="B17" s="29">
+        <v>16</v>
+      </c>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="29"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" s="28"/>
+      <c r="B18" s="29">
+        <v>17</v>
+      </c>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="29"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1623,288 +2400,1165 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19F63B13-47E9-468A-80A4-B58BA6E90505}">
-  <dimension ref="A1:P9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2225A231-F8A8-4742-9726-359A721358A8}">
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.36328125" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.7265625" style="10"/>
-    <col min="3" max="3" width="18.81640625" style="10" customWidth="1"/>
-    <col min="4" max="4" width="16.6328125" style="10" customWidth="1"/>
-    <col min="5" max="5" width="11.54296875" style="10" customWidth="1"/>
-    <col min="6" max="6" width="11.6328125" style="10" customWidth="1"/>
-    <col min="7" max="7" width="10.90625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="10.7265625" style="10" customWidth="1"/>
-    <col min="9" max="9" width="10.90625" style="10" customWidth="1"/>
-    <col min="10" max="11" width="11" style="10" customWidth="1"/>
-    <col min="12" max="12" width="10.08984375" style="10" customWidth="1"/>
-    <col min="13" max="13" width="11.08984375" style="10" customWidth="1"/>
-    <col min="14" max="14" width="10.90625" style="10" customWidth="1"/>
-    <col min="15" max="15" width="12" style="10" customWidth="1"/>
-    <col min="16" max="16" width="9.7265625" style="10" customWidth="1"/>
-    <col min="17" max="16384" width="8.7265625" style="10"/>
+    <col min="1" max="1" width="10.7265625" style="9" customWidth="1"/>
+    <col min="2" max="4" width="10.7265625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="30.6328125" style="7" customWidth="1"/>
+    <col min="6" max="6" width="19.54296875" style="7" customWidth="1"/>
+    <col min="7" max="7" width="13.7265625" style="7" customWidth="1"/>
+    <col min="8" max="8" width="35" style="7" customWidth="1"/>
+    <col min="9" max="9" width="17.26953125" style="7" customWidth="1"/>
+    <col min="10" max="16384" width="8.7265625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="C1" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="26" t="s">
+      <c r="C1" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="H1" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="I1" s="26" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="29">
         <v>1</v>
       </c>
+      <c r="C2" s="1">
+        <v>949</v>
+      </c>
+      <c r="D2" s="1"/>
+      <c r="E2" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="1">
+        <v>12345</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="1">
+        <v>12345</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="8"/>
+      <c r="B3" s="29">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="1">
+        <v>12345</v>
+      </c>
+      <c r="G3" s="1"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="28"/>
+      <c r="B4" s="29">
+        <v>3</v>
+      </c>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="29"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="28"/>
+      <c r="B5" s="29">
+        <v>4</v>
+      </c>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="29"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="28"/>
+      <c r="B6" s="29">
+        <v>5</v>
+      </c>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="29"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="28"/>
+      <c r="B7" s="29">
+        <v>6</v>
+      </c>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="29"/>
+      <c r="H7" s="29"/>
+      <c r="I7" s="29"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="28"/>
+      <c r="B8" s="29">
+        <v>7</v>
+      </c>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="29"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="28"/>
+      <c r="B9" s="29">
+        <v>8</v>
+      </c>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="29"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="28"/>
+      <c r="B10" s="29">
+        <v>9</v>
+      </c>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="28"/>
+      <c r="B11" s="29">
+        <v>10</v>
+      </c>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="29"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="28"/>
+      <c r="B12" s="29">
+        <v>11</v>
+      </c>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="29"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" s="28"/>
+      <c r="B13" s="29">
+        <v>12</v>
+      </c>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" s="28"/>
+      <c r="B14" s="29">
+        <v>13</v>
+      </c>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="29"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="28"/>
+      <c r="B15" s="29">
+        <v>14</v>
+      </c>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="29"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="28"/>
+      <c r="B16" s="29">
+        <v>15</v>
+      </c>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="29"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" s="28"/>
+      <c r="B17" s="29">
+        <v>16</v>
+      </c>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="29"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" s="28"/>
+      <c r="B18" s="29">
+        <v>17</v>
+      </c>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="29"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AA46238-0993-45CC-A6AB-36332C11875C}">
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.7265625" style="9" customWidth="1"/>
+    <col min="2" max="4" width="10.7265625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="30.6328125" style="7" customWidth="1"/>
+    <col min="6" max="6" width="19.54296875" style="7" customWidth="1"/>
+    <col min="7" max="7" width="13.7265625" style="7" customWidth="1"/>
+    <col min="8" max="8" width="35" style="7" customWidth="1"/>
+    <col min="9" max="9" width="17.26953125" style="7" customWidth="1"/>
+    <col min="10" max="16384" width="8.7265625" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>68</v>
+      </c>
       <c r="E1" s="26" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="F1" s="26" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="G1" s="26" t="s">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="H1" s="26" t="s">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="I1" s="26" t="s">
-        <v>74</v>
-      </c>
-      <c r="J1" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="K1" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="L1" s="26" t="s">
-        <v>88</v>
-      </c>
-      <c r="M1" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="N1" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="O1" s="26" t="s">
-        <v>100</v>
-      </c>
-      <c r="P1" s="26" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" ht="174" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="29">
         <v>1</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="1">
+        <v>950</v>
+      </c>
+      <c r="D2" s="1"/>
+      <c r="E2" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="1">
+        <v>12345</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="1">
+        <v>12345</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="8"/>
+      <c r="B3" s="29">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="1">
+        <v>12345</v>
+      </c>
+      <c r="G3" s="1"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="28"/>
+      <c r="B4" s="29">
+        <v>3</v>
+      </c>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="29"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="28"/>
+      <c r="B5" s="29">
+        <v>4</v>
+      </c>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="29"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="28"/>
+      <c r="B6" s="29">
         <v>5</v>
       </c>
-      <c r="D2" s="9">
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="29"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="28"/>
+      <c r="B7" s="29">
+        <v>6</v>
+      </c>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="29"/>
+      <c r="H7" s="29"/>
+      <c r="I7" s="29"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="28"/>
+      <c r="B8" s="29">
+        <v>7</v>
+      </c>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="29"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="28"/>
+      <c r="B9" s="29">
+        <v>8</v>
+      </c>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="29"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="28"/>
+      <c r="B10" s="29">
+        <v>9</v>
+      </c>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="28"/>
+      <c r="B11" s="29">
+        <v>10</v>
+      </c>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="29"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="28"/>
+      <c r="B12" s="29">
+        <v>11</v>
+      </c>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="29"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" s="28"/>
+      <c r="B13" s="29">
+        <v>12</v>
+      </c>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" s="28"/>
+      <c r="B14" s="29">
+        <v>13</v>
+      </c>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="29"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="28"/>
+      <c r="B15" s="29">
+        <v>14</v>
+      </c>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="29"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="28"/>
+      <c r="B16" s="29">
+        <v>15</v>
+      </c>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="29"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" s="28"/>
+      <c r="B17" s="29">
+        <v>16</v>
+      </c>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="29"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" s="28"/>
+      <c r="B18" s="29">
+        <v>17</v>
+      </c>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="29"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A171683-70E2-41CC-B93D-30B4C5358BCB}">
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.7265625" style="9" customWidth="1"/>
+    <col min="2" max="4" width="10.7265625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="30.6328125" style="7" customWidth="1"/>
+    <col min="6" max="6" width="19.54296875" style="7" customWidth="1"/>
+    <col min="7" max="7" width="13.7265625" style="7" customWidth="1"/>
+    <col min="8" max="8" width="35" style="7" customWidth="1"/>
+    <col min="9" max="9" width="17.26953125" style="7" customWidth="1"/>
+    <col min="10" max="16384" width="8.7265625" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="H1" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="I1" s="26" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="29">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1">
+        <v>949</v>
+      </c>
+      <c r="D2" s="1"/>
+      <c r="E2" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="1">
         <v>12345</v>
       </c>
-      <c r="E2" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="J2" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="K2" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="L2" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="M2" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="N2" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="O2" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="P2" s="9" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" ht="87" x14ac:dyDescent="0.35">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9">
+      <c r="G2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="1">
+        <v>12345</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="8"/>
+      <c r="B3" s="29">
         <v>2</v>
       </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="L3" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="M3" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A4" s="27"/>
-      <c r="B4" s="27">
+      <c r="C3" s="1"/>
+      <c r="D3" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="1">
+        <v>12345</v>
+      </c>
+      <c r="G3" s="1"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="28"/>
+      <c r="B4" s="29">
         <v>3</v>
       </c>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
-      <c r="K4" s="27"/>
-      <c r="L4" s="27"/>
-      <c r="M4" s="27"/>
-      <c r="N4" s="27"/>
-      <c r="O4" s="27"/>
-      <c r="P4" s="27"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A5" s="9"/>
-      <c r="B5" s="9">
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="29"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="28"/>
+      <c r="B5" s="29">
         <v>4</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
-      <c r="N5" s="9"/>
-      <c r="O5" s="9"/>
-      <c r="P5" s="9"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A6" s="9"/>
-      <c r="B6" s="9">
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="29"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="28"/>
+      <c r="B6" s="29">
         <v>5</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="9"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9">
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="29"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="28"/>
+      <c r="B7" s="29">
         <v>6</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="9"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9">
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="29"/>
+      <c r="H7" s="29"/>
+      <c r="I7" s="29"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="28"/>
+      <c r="B8" s="29">
         <v>7</v>
       </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9">
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="29"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="28"/>
+      <c r="B9" s="29">
         <v>8</v>
       </c>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="9"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="29"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="28"/>
+      <c r="B10" s="29">
+        <v>9</v>
+      </c>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="28"/>
+      <c r="B11" s="29">
+        <v>10</v>
+      </c>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="29"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="28"/>
+      <c r="B12" s="29">
+        <v>11</v>
+      </c>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="29"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" s="28"/>
+      <c r="B13" s="29">
+        <v>12</v>
+      </c>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" s="28"/>
+      <c r="B14" s="29">
+        <v>13</v>
+      </c>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="29"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="28"/>
+      <c r="B15" s="29">
+        <v>14</v>
+      </c>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="29"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="28"/>
+      <c r="B16" s="29">
+        <v>15</v>
+      </c>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="29"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" s="28"/>
+      <c r="B17" s="29">
+        <v>16</v>
+      </c>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="29"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" s="28"/>
+      <c r="B18" s="29">
+        <v>17</v>
+      </c>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="29"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C5EDADE-53D7-4DF0-A23E-AEF5DB73204D}">
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.7265625" style="9" customWidth="1"/>
+    <col min="2" max="4" width="10.7265625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="30.6328125" style="7" customWidth="1"/>
+    <col min="6" max="6" width="19.54296875" style="7" customWidth="1"/>
+    <col min="7" max="7" width="13.7265625" style="7" customWidth="1"/>
+    <col min="8" max="8" width="35" style="7" customWidth="1"/>
+    <col min="9" max="9" width="17.26953125" style="7" customWidth="1"/>
+    <col min="10" max="16384" width="8.7265625" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="H1" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="I1" s="26" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="29">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1">
+        <v>950</v>
+      </c>
+      <c r="D2" s="1"/>
+      <c r="E2" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="1">
+        <v>12345</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="1">
+        <v>12345</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="8"/>
+      <c r="B3" s="29">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="1">
+        <v>12345</v>
+      </c>
+      <c r="G3" s="1"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="28"/>
+      <c r="B4" s="29">
+        <v>3</v>
+      </c>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="29"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="28"/>
+      <c r="B5" s="29">
+        <v>4</v>
+      </c>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="29"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="28"/>
+      <c r="B6" s="29">
+        <v>5</v>
+      </c>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="29"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="28"/>
+      <c r="B7" s="29">
+        <v>6</v>
+      </c>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="29"/>
+      <c r="H7" s="29"/>
+      <c r="I7" s="29"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="28"/>
+      <c r="B8" s="29">
+        <v>7</v>
+      </c>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="29"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="28"/>
+      <c r="B9" s="29">
+        <v>8</v>
+      </c>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="29"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="28"/>
+      <c r="B10" s="29">
+        <v>9</v>
+      </c>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="28"/>
+      <c r="B11" s="29">
+        <v>10</v>
+      </c>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="29"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="28"/>
+      <c r="B12" s="29">
+        <v>11</v>
+      </c>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="29"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" s="28"/>
+      <c r="B13" s="29">
+        <v>12</v>
+      </c>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" s="28"/>
+      <c r="B14" s="29">
+        <v>13</v>
+      </c>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="29"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="28"/>
+      <c r="B15" s="29">
+        <v>14</v>
+      </c>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="29"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="28"/>
+      <c r="B16" s="29">
+        <v>15</v>
+      </c>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="29"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" s="28"/>
+      <c r="B17" s="29">
+        <v>16</v>
+      </c>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="29"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" s="28"/>
+      <c r="B18" s="29">
+        <v>17</v>
+      </c>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="29"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Script Fixed and Updated
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C4B41B8-9157-4F3E-9588-DD26EE062DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69582505-33EC-4208-966C-47F1837F75A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="720" windowWidth="17610" windowHeight="8570" tabRatio="902" firstSheet="5" activeTab="6" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
+    <workbookView xWindow="720" yWindow="720" windowWidth="17610" windowHeight="8570" tabRatio="902" firstSheet="6" activeTab="9" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
   <sheets>
     <sheet name="BrowserSetup" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="101">
   <si>
     <t>Username</t>
   </si>
@@ -1077,7 +1077,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>951</v>
+        <v>959</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="32" t="s">
@@ -2159,7 +2159,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>946</v>
+        <v>953</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="18" t="s">
@@ -2433,15 +2433,9 @@
       <c r="F1" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="H1" s="26" t="s">
-        <v>43</v>
-      </c>
-      <c r="I1" s="26" t="s">
-        <v>44</v>
-      </c>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
@@ -2451,7 +2445,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="18" t="s">
@@ -2460,15 +2454,9 @@
       <c r="F2" s="1">
         <v>12345</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="H2" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="I2" s="1">
-        <v>12345</v>
-      </c>
+      <c r="G2" s="1"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="1"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="8"/>
@@ -2742,7 +2730,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>950</v>
+        <v>956</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="18" t="s">
@@ -3033,7 +3021,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>949</v>
+        <v>957</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="18" t="s">
@@ -3324,7 +3312,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>950</v>
+        <v>958</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="18" t="s">

</xml_diff>

<commit_message>
Script Optimized and Updated
</commit_message>
<xml_diff>
--- a/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
+++ b/GlideGo_WebAutomation_BDD/Resources/TestData/GlideGoWebData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohai\source\repos\GlideGo_WebAutomation_BDD\GlideGo_WebAutomation_BDD\Resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69582505-33EC-4208-966C-47F1837F75A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F268A02A-79BC-4F45-8FE1-0B33B4D3CF11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="720" yWindow="720" windowWidth="17610" windowHeight="8570" tabRatio="902" firstSheet="6" activeTab="9" xr2:uid="{C3258C78-C11E-4EE3-87DC-9D54192C14DE}"/>
   </bookViews>
@@ -1077,7 +1077,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>959</v>
+        <v>971</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="32" t="s">
@@ -2159,7 +2159,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>953</v>
+        <v>966</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="18" t="s">
@@ -2445,7 +2445,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>955</v>
+        <v>967</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="18" t="s">
@@ -2730,7 +2730,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>956</v>
+        <v>968</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="18" t="s">
@@ -3021,7 +3021,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>957</v>
+        <v>969</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="18" t="s">
@@ -3312,7 +3312,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>958</v>
+        <v>970</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="18" t="s">

</xml_diff>